<commit_message>
Completar matriz con lectura de providencias del nivel A (reglas, citas y resultados)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HFz41Xq5pxE4jPsKEtG9Mg
</commit_message>
<xml_diff>
--- a/Matriz_Valoracion_Probatoria_Disciplinaria.xlsx
+++ b/Matriz_Valoracion_Probatoria_Disciplinaria.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matriz'!$A$1:$J$260</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matriz'!$A$1:$L$260</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J260"/>
+  <dimension ref="A1:L260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -442,8 +442,10 @@
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="90" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -494,14 +496,24 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Regla / problema jurídico (pendiente)</t>
+          <t>Regla / problema jurídico (cita textual)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Resultado (decisión)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Términos hallados en el texto (n.º de apariciones)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>A – título señala tema probatorio</t>
+          <t>A1 – verificada, central</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -541,19 +553,29 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí – lectura dirigida</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Num. 7.3, «La prueba del dolo»: su prueba «radica en la demostración de hechos subjetivos»; los medios son la confesión y «la prueba indiciaria, que no es más que “la aplicación por parte del juez de determinadas máximas de la experiencia a hechos de naturaleza objetiva previamente probados”». Desarrolla la «teoría de los dos niveles de valoración» (convicción ajustada a la lógica, la experiencia y el conocimiento científico).</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Revoca la sentencia de primera instancia que había sancionado al abogado con suspensión (Ley 1123 de 2007). Lectura parcial del resuelve (texto truncado en la extracción).</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>prueba indiciaria / indicios (3)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>A – título señala tema probatorio</t>
+          <t>A1 – verificada, central</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -563,101 +585,121 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>11001-11-02-000-2019-07466-01</t>
+          <t>41001250200020210023502</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>25-10-2024</t>
+          <t>27-11-2024</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>CNDJ – Rad. 11001-11-02-000-2019-07466-01 – Exclusion de la profesion por ejercer estando suspendido</t>
+          <t>CNDJ – Rad. 41001250200020210023502 – Principio de investigación integral</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>apreciación probatoria</t>
+          <t>apreciación probatoria; sana crítica; valoración probatoria</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1T4ZizI1hcgg2OI4GpHy67qErDEC6_kGh/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/19R41xVH1s6L6ndCO8ILZO0HnRyPj9j2Z/view?usp=drivesdk</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>1T4ZizI1hcgg2OI4GpHy67qErDEC6_kGh</t>
+          <t>19R41xVH1s6L6ndCO8ILZO0HnRyPj9j2Z</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí – lectura dirigida</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Investigación integral (art. 13 Ley 1952/2019) y mensajes de voz de WhatsApp. Citando T-561/2005: «el juez al realizar la valoración de la prueba, lo que ha de realizar conforme a las reglas de la sana crítica, debe llegar a la certeza o convicción sobre la existencia del hecho y la culpabilidad». Sobre autenticidad (art. 11 Ley 527/1999): «no es cierto que porque se tengan dudas sobre la identificación del iniciador de las pruebas documentales aportadas por el quejoso se reputen como ilegales. En contraposición, le corresponde al juzgador disciplinario considerar los aspectos allí contenidos para delimitar su fuerza probatoria». Reprocha no haber acudido a pruebas técnicas para establecer si la voz era de la disciplinada.</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Revoca parcialmente el auto de terminación (empleada judicial); ordena continuar la investigación por la presunta asesoría; confirma en lo demás.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>sana crítica (2); referencias a prueba lícita/ilícita de mensajes de voz (lectura completa)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>A – título señala tema probatorio</t>
+          <t>A1 – verificada, central</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Comisión Nacional de Disciplina Judicial</t>
+          <t>Consejo de Estado – Sec. 2ª</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>41001250200020210023502</t>
+          <t>50001-23-33-000-2014-00058-01</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>27-11-2024</t>
+          <t>06-06-2019</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>CNDJ – Rad. 41001250200020210023502 – Principio de investigación integral</t>
+          <t>CE Secc. 2ª – Rad. 50001-23-33-000-2014-00058-01 (1144-16) – Sancion disciplinaria policia embriaguez en servicio prueba alcoholemia</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>apreciación probatoria; sana crítica; valoración probatoria</t>
+          <t>apreciación probatoria; prueba ilícita; valoración probatoria</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/19R41xVH1s6L6ndCO8ILZO0HnRyPj9j2Z/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ILgJgVvcl6F9FGztX7VjJ-fIQE657C_X/view?usp=drivesdk</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>19R41xVH1s6L6ndCO8ILZO0HnRyPj9j2Z</t>
+          <t>1ILgJgVvcl6F9FGztX7VjJ-fIQE657C_X</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí – lectura dirigida</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Reseña: «El examen de alcoholemia practicado por el Instituto de Medicina Legal no es la única prueba idónea para que se tipifique la falta contenida en el artículo 34 numeral 26 de la Ley 1015 de 2006, pues son admisibles otros medios de convicción». Falta acreditada «más allá de toda duda razonable» con minutas de guardia, anotaciones y testimonios. También: en la indagación preliminar el titular «no tiene la obligación de realizar una valoración probatoria previa».</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Confirma la sentencia que denegó las pretensiones (policía sancionado por presentarse al servicio bajo efectos del alcohol).</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>valoración probatoria (2), indicios (3)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>A – título señala tema probatorio</t>
+          <t>A1 – verificada, central</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -667,49 +709,59 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>11001-03-25-000-2014-00400-00</t>
+          <t>11001-03-25-000-2011-00574-00</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>14-03-2019</t>
+          <t>25-11-2021</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>CE Secc. 2ª – Rad. 11001-03-25-000-2014-00400-00 (1270-14) – Nulidad destitucion Directora Investigaciones Especiales PGN interceptaciones</t>
+          <t>CE Secc. 2ª – Rad. 11001-03-25-000-2011-00574-00 (2201-11) – Exclusión probatoria de grabación magnetofónica y autonomía disciplinaria</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>apreciación probatoria; sana crítica; valoración probatoria</t>
+          <t>apreciación probatoria; prueba ilícita; valoración probatoria</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1siAQrcdMK7qKte6mwClmSgJGcZ-Y-kcf/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1XC4DvvMLkAEZWEbaginl3s-JJOWA_RGx/view?usp=drivesdk</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>1siAQrcdMK7qKte6mwClmSgJGcZ-Y-kcf</t>
+          <t>1XC4DvvMLkAEZWEbaginl3s-JJOWA_RGx</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí – lectura dirigida</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Cláusula de exclusión del art. 29 C.P.: «tienen como fuente de exclusión la obtención de la prueba mediante la vulneración del núcleo esencial de un derecho fundamental -prueba inconstitucional-, así como el desconocimiento de las condiciones legales y/o requisitos sustanciales específicos para la práctica de cada prueba en particular –prueba ilegal-, teniendo como consecuencia que aquella no pueda ser valorada ni usada para sustentar una decisión en derecho». Aplica por el art. 21 Ley 734 las excepciones de la regla (vínculo atenuado, fuente independiente, descubrimiento inevitable) y la regla de que la víctima puede grabar sin autorización judicial.</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Niega las pretensiones (destitución e inhabilidad 12 años a Representante a la Cámara); la grabación se tuvo por válida con cadena de custodia y pericia.</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>prueba ilícita / exclusión (16), valoración probatoria (5), apreciación probatoria (1)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>A – título señala tema probatorio</t>
+          <t>A1 – verificada, central</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -719,49 +771,59 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>50001-23-33-000-2014-00058-01</t>
+          <t>66001-23-33-000-2015-00369-01</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>06-06-2019</t>
+          <t>13-04-2023</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>CE Secc. 2ª – Rad. 50001-23-33-000-2014-00058-01 (1144-16) – Sancion disciplinaria policia embriaguez en servicio prueba alcoholemia</t>
+          <t>CE Secc. 2ª – Rad. 66001-23-33-000-2015-00369-01 (4344-2018) – Sanción disciplinaria, adecuación típica y presunción de inocencia</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>apreciación probatoria; prueba ilícita; valoración probatoria</t>
+          <t>apreciación probatoria; prueba ilícita; prueba indiciaria; sana crítica; valoración probatoria</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ILgJgVvcl6F9FGztX7VjJ-fIQE657C_X/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1wme2tgsgeCNsYtuuBjNDbL37NmHLZtP8/view?usp=drivesdk</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>1ILgJgVvcl6F9FGztX7VjJ-fIQE657C_X</t>
+          <t>1wme2tgsgeCNsYtuuBjNDbL37NmHLZtP8</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí – lectura dirigida</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Párr. 117: «la autoridad disciplinaria en el momento de emitir la decisión condenatoria debe tener la convicción y la certeza probatoria de que efectivamente el servidor público incurrió en la falta que se le imputa. La existencia de dudas al respecto implica necesariamente que estas se resuelvan en favor del investigado». Indicios: las fotografías del álbum «son muy borrosas y por sí mismas no permiten establecer con certeza que los interlocutores de la conversación son los demandantes […] por lo que tal documental no puede ser apreciada como indicio» (párr. 135); «los indicios […] no pueden dar por configurada la tipicidad de la conducta» (párr. 138).</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Confirma la sentencia que accedió parcialmente a las pretensiones (policías sancionados por hurto de celulares); condena en costas a la demandada.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>indicios (20), sana crítica (4), valoración probatoria (5), prueba ilícita (1)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>A – título señala tema probatorio</t>
+          <t>A1 – verificada, central</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -771,49 +833,59 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>25000-23-42-000-2013-06021-01</t>
+          <t>76001-23-33-000-2014-00504-01</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>06-02-2020</t>
+          <t>15-06-2023</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>CE Secc. 2ª – Rad. 25000-23-42-000-2013-06021-01 (3003-17) – Estructura dogmatica ilicitud sustancial y culpabilidad disciplinaria</t>
+          <t>CE Secc. 2ª – Rad. 76001-23-33-000-2014-00504-01 (1667-2022) – Certeza probatoria en sancion disciplinaria policial y absolucion penal</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>apreciación probatoria; valoración probatoria</t>
+          <t>apreciación probatoria; prueba trasladada; sana crítica; valoración probatoria</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1LDpqSquUReB9IDEyJkt969hvZVtDb_rW/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/11vKHDPRYh1Buuul51URtWC3GXpvUTecW/view?usp=drivesdk</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>1LDpqSquUReB9IDEyJkt969hvZVtDb_rW</t>
+          <t>11vKHDPRYh1Buuul51URtWC3GXpvUTecW</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí – lectura dirigida</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Citando arts. 140 y 142 Ley 734 de 2002: «Las pruebas deberán apreciarse conjuntamente, de acuerdo con las reglas de la sana crítica»; no se puede sancionar «sin que obre en el proceso prueba que conduzca a la certeza sobre la existencia de la falta y de la responsabilidad del investigado». Autonomía de la acción disciplinaria: «no implica, en modo alguno, que en este caso se admitan como ciertos los delitos que la justicia penal demostró que el demandante no cometió». Critica que el a quo no hizo «análisis crítico de las pruebas» (art. 187 CPACA).</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Revoca parcialmente la sentencia; nulidad parcial de la destitución e inhabilidad general de 20 años del patrullero; ordena restablecimiento.</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>sana crítica (3), prueba trasladada (1)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>A – título señala tema probatorio</t>
+          <t>A1 – verificada, central</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -823,49 +895,59 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>11001-03-25-000-2011-00574-00</t>
+          <t>52001-23-33-000-2014-00562-02</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>25-11-2021</t>
+          <t>11-04-2024</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>CE Secc. 2ª – Rad. 11001-03-25-000-2011-00574-00 (2201-11) – Exclusión probatoria de grabación magnetofónica y autonomía disciplinaria</t>
+          <t>CE Secc. 2ª – Rad. 52001-23-33-000-2014-00562-02 (4923-2022) – Nulidad sancion disciplinaria destitucion docente valoracion probatoria</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>apreciación probatoria; prueba ilícita; valoración probatoria</t>
+          <t>sana crítica; valoración probatoria</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1XC4DvvMLkAEZWEbaginl3s-JJOWA_RGx/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1oVC8hzyUGv8RaczXOPe-MMl6K-ra_D7E/view?usp=drivesdk</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>1XC4DvvMLkAEZWEbaginl3s-JJOWA_RGx</t>
+          <t>1oVC8hzyUGv8RaczXOPe-MMl6K-ra_D7E</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí – lectura dirigida</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Control integral (tipicidad, ilicitud, culpabilidad, proporcionalidad y valoración probatoria). Valoración de testimonios de menores y de CD aportado con la queja; aplica sana crítica a la prueba testimonial («en el análisis de la prueba testimonial, es donde deben utilizarse con mayor rigor las reglas de la sana crítica», pasaje citado en la sentencia). Concluye: «el testimonio de los menores no era la única prueba obrante en el proceso» y «existió un adecuado examen de los dichos de los declarantes».</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Confirma parcialmente la sentencia que negó la nulidad (destitución e inhabilidad a docente); revoca la condena en costas.</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>valoración probatoria (1), sana crítica (2), prueba ilícita (1), indicios (1)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>A – título señala tema probatorio</t>
+          <t>A1 – verificada, central</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -875,101 +957,117 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>66001-23-33-000-2015-00369-01</t>
+          <t>11001-03-25-000-2014-00034-00</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>13-04-2023</t>
+          <t>20-06-2024</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>CE Secc. 2ª – Rad. 66001-23-33-000-2015-00369-01 (4344-2018) – Sanción disciplinaria, adecuación típica y presunción de inocencia</t>
+          <t>CE Secc. 2ª – Rad. 11001-03-25-000-2014-00034-00 (0086-2014) – Nulidad sancion disciplinaria contralor Barranquilla prueba trasladada penal</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>apreciación probatoria; prueba ilícita; prueba indiciaria; sana crítica; valoración probatoria</t>
+          <t>prueba trasladada; valoración probatoria</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1wme2tgsgeCNsYtuuBjNDbL37NmHLZtP8/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1d2Xt9PhFwY9OHgq6zGyTmYuk1WTojGxA/view?usp=drivesdk</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>1wme2tgsgeCNsYtuuBjNDbL37NmHLZtP8</t>
+          <t>1d2Xt9PhFwY9OHgq6zGyTmYuk1WTojGxA</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí – lectura dirigida</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Defecto fáctico por indebida obtención de la prueba (dimensión positiva). «estos informes no constituían prueba en sí mismos porque, como ya se vio, se practicaron fuera del juicio al haberse recolectado en la etapa de indagación, por lo que no podían introducirse al proceso disciplinario como “prueba trasladada”, en la medida que no fueron decretados, practicados ni controvertidos en sede penal». Los actos «incorporaron como pruebas y única fuente de motivación, documentos que no revestían dicha calidad». Régimen: art. 135 Ley 734 (mod. art. 51 Ley 1474/2011).</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Anula el fallo de única instancia (destitución e inhabilidad 12 años, contralor distrital) y el que lo confirmó; ordena eliminar el registro; niega perjuicios morales por falta de prueba.</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>prueba trasladada, sana crítica, valoración probatoria (lectura completa)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>A – título señala tema probatorio</t>
+          <t>A1 – verificada, central</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Consejo de Estado – Sec. 2ª</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>76001-23-33-000-2014-00504-01</t>
-        </is>
-      </c>
+          <t>Corte Constitucional</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>15-06-2023</t>
+          <t>22-01-2025</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>CE Secc. 2ª – Rad. 76001-23-33-000-2014-00504-01 (1667-2022) – Certeza probatoria en sancion disciplinaria policial y absolucion penal</t>
+          <t>CC – Sentencia T-013-25 – Defecto factico por indebida valoracion probatoria proceso disciplinario abogado</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>apreciación probatoria; prueba trasladada; sana crítica; valoración probatoria</t>
+          <t>apreciación probatoria; sana crítica; valoración probatoria</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/11vKHDPRYh1Buuul51URtWC3GXpvUTecW/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1u-B90hluuySWAaGldP6aqmgThzGfRpS2/view?usp=drivesdk</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>11vKHDPRYh1Buuul51URtWC3GXpvUTecW</t>
+          <t>1u-B90hluuySWAaGldP6aqmgThzGfRpS2</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí – lectura dirigida</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Defecto fáctico en tutela contra decisión de la CNDJ (proceso disciplinario de abogado). Párr. 199: «para que se configure este defecto no basta una diferencia de criterio en la apreciación de las pruebas, sino que el juez debe haber omitido completamente la valoración de medios probatorios que eran relevantes para la decisión o su valoración debe ser manifiestamente irracional, fuera de toda lógica o incumplir estándares legales de valoración probatoria cuando estos existan». Párr. 206: los jueces disciplinarios «omitieron decretar las pruebas indispensables para demostrar la existencia o inexistencia de estos hechos relevantes».</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Concede la tutela; deja sin efecto el cierre anticipado (art. 103 Ley 1123 de 2007) y ordena retomar la actuación y formular cargos.</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>valoración probatoria (4), sana crítica (2)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>A – título señala tema probatorio</t>
+          <t>A2 – verificada, tangencial (lectura parcial)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -979,49 +1077,59 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>11001-03-25-000-2012-00817-00</t>
+          <t>11001-03-25-000-2014-00400-00</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>15-02-2024</t>
+          <t>14-03-2019</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>CE Secc. 2ª – Rad. 11001-03-25-000-2012-00817-00 (2592-2012) – Nulidad sancion disciplinaria PGN subdirectora DAS chuzadas</t>
+          <t>CE Secc. 2ª – Rad. 11001-03-25-000-2014-00400-00 (1270-14) – Nulidad destitucion Directora Investigaciones Especiales PGN interceptaciones</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>valoración probatoria</t>
+          <t>apreciación probatoria; sana crítica; valoración probatoria</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1K9DNjDMhiQV3KkwuVPR0L9-ULfepILKQ/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1siAQrcdMK7qKte6mwClmSgJGcZ-Y-kcf/view?usp=drivesdk</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>1K9DNjDMhiQV3KkwuVPR0L9-ULfepILKQ</t>
+          <t>1siAQrcdMK7qKte6mwClmSgJGcZ-Y-kcf</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí – lectura dirigida</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sanción a directora de investigaciones especiales de la PGN por solicitar interceptaciones. El sumario señala los requisitos de la interceptación: «orden judicial previa, fundamentada por escrito», bajo dirección del Procurador General. La sentencia da por cumplidos esos requisitos; el fundamento de la nulidad no se verificó en esta lectura.</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Declara la nulidad de los actos sancionatorios; ordena eliminar el antecedente y reconoce perjuicios (moral y material por pérdida de oportunidad).</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>valoración probatoria (1), sana crítica (2), indicios (1)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>A – título señala tema probatorio</t>
+          <t>A2 – verificada, tangencial</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1031,49 +1139,59 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>52001-23-33-000-2014-00562-02</t>
+          <t>25000-23-42-000-2013-06021-01</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>11-04-2024</t>
+          <t>06-02-2020</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>CE Secc. 2ª – Rad. 52001-23-33-000-2014-00562-02 (4923-2022) – Nulidad sancion disciplinaria destitucion docente valoracion probatoria</t>
+          <t>CE Secc. 2ª – Rad. 25000-23-42-000-2013-06021-01 (3003-17) – Estructura dogmatica ilicitud sustancial y culpabilidad disciplinaria</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>sana crítica; valoración probatoria</t>
+          <t>apreciación probatoria; valoración probatoria</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1oVC8hzyUGv8RaczXOPe-MMl6K-ra_D7E/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1LDpqSquUReB9IDEyJkt969hvZVtDb_rW/view?usp=drivesdk</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>1oVC8hzyUGv8RaczXOPe-MMl6K-ra_D7E</t>
+          <t>1LDpqSquUReB9IDEyJkt969hvZVtDb_rW</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí – lectura dirigida</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Tema central: estructura dogmática de la responsabilidad (tipicidad, ilicitud sustancial, culpabilidad). Solo reitera de la unificación de 2016 que «la interpretación normativa y la valoración probatoria hecha en sede disciplinaria, es controlable judicialmente».</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Revoca la sentencia de primera instancia y deniega las pretensiones; condena en costas al demandante.</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>valoración probatoria (2), indicios (12; uso no verificado)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>A – título señala tema probatorio</t>
+          <t>A2 – verificada, tangencial</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1083,194 +1201,238 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>11001-03-25-000-2014-00034-00</t>
+          <t>11001-03-25-000-2012-00817-00</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>20-06-2024</t>
+          <t>15-02-2024</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>CE Secc. 2ª – Rad. 11001-03-25-000-2014-00034-00 (0086-2014) – Nulidad sancion disciplinaria contralor Barranquilla prueba trasladada penal</t>
+          <t>CE Secc. 2ª – Rad. 11001-03-25-000-2012-00817-00 (2592-2012) – Nulidad sancion disciplinaria PGN subdirectora DAS chuzadas</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>prueba trasladada; valoración probatoria</t>
+          <t>valoración probatoria</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1d2Xt9PhFwY9OHgq6zGyTmYuk1WTojGxA/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1K9DNjDMhiQV3KkwuVPR0L9-ULfepILKQ/view?usp=drivesdk</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>1d2Xt9PhFwY9OHgq6zGyTmYuk1WTojGxA</t>
+          <t>1K9DNjDMhiQV3KkwuVPR0L9-ULfepILKQ</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí – lectura dirigida</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>El fallo disciplinario se apoyó en correos, actas, declaraciones, versión libre y prueba trasladada (disco duro y otros procesos IUC). El análisis central es de tipicidad y congruencia con las pruebas; no se encontró una regla autónoma sobre valoración o traslado.</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Niega las pretensiones (subdirectora de operaciones del DAS); sin costas.</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>prueba trasladada (5), valoración probatoria (1)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>A – título señala tema probatorio</t>
+          <t>A2 – verificada, tangencial</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Corte Constitucional</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr"/>
+          <t>Corte Suprema de Justicia</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>68644</t>
+        </is>
+      </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>22-01-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>CC – Sentencia T-013-25 – Defecto factico por indebida valoracion probatoria proceso disciplinario abogado</t>
+          <t>CSJ Sala Penal – Rad. 68644 (AP2765-2025) – Impertinencia de fallo disciplinario como prueba en juicio penal prevaricato</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>apreciación probatoria; sana crítica; valoración probatoria</t>
+          <t>prueba trasladada; valoración probatoria</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1u-B90hluuySWAaGldP6aqmgThzGfRpS2/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/13lHxg1-YXa7pW6ay6khkzQqpllYn8mlE/view?usp=drivesdk</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>1u-B90hluuySWAaGldP6aqmgThzGfRpS2</t>
+          <t>13lHxg1-YXa7pW6ay6khkzQqpllYn8mlE</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí – lectura dirigida</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No trata la valoración probatoria en sede disciplinaria sino la pertinencia de un fallo disciplinario como prueba en juicio penal. Párr. 49: «las decisiones disciplinarias (o fiscales) reflejan la valoración de las pruebas allí practicadas, que no tienen la entidad para imponerse o incidir en la actuación penal, así se trate de los mismos supuestos fácticos o jurídicos». Cita CSJ AP 30-sep-2015, rad. 46153: «en el sistema reglado en la Ley 906 de 2004 no opera la figura de la prueba trasladada».</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Confirma la negativa a decretar la sentencia disciplinaria y el testimonio del secretario como pruebas de la defensa (juez acusado de prevaricato).</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>prueba trasladada (cita de doctrina de la Sala), valoración</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>A – título señala tema probatorio</t>
+          <t>A2 – verificada, tangencial</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Corte Suprema de Justicia</t>
+          <t>Tribunal Administrativo</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>68644</t>
+          <t>25000-23-42-000-2016-02740-01</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>31-10-2024</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>CSJ Sala Penal – Rad. 68644 (AP2765-2025) – Impertinencia de fallo disciplinario como prueba en juicio penal prevaricato</t>
+          <t>TA Cundinamarca – Rad. 25000-23-42-000-2016-02740-01 – Nulidad y restablecimiento sancion disciplinaria policial culpa grave frente a dolo</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>prueba trasladada; valoración probatoria</t>
+          <t>apreciación probatoria; sana crítica; valoración probatoria</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/13lHxg1-YXa7pW6ay6khkzQqpllYn8mlE/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1_1OrQcyc38GEWJits46ul3-95g66AeIo/view?usp=drivesdk</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>13lHxg1-YXa7pW6ay6khkzQqpllYn8mlE</t>
+          <t>1_1OrQcyc38GEWJits46ul3-95g66AeIo</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí – lectura dirigida</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Tema central: culpa grave frente a dolo. Reitera que el control judicial debe ser integral, incluyendo «la valoración fáctica, probatoria (conforme a las reglas de la sana crítica)».</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Accede parcialmente a las pretensiones (policial sancionada con destitución).</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>valoración probatoria (2), sana crítica (2)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>A – título señala tema probatorio</t>
+          <t>D – descartada</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Tribunal Administrativo</t>
+          <t>Comisión Nacional de Disciplina Judicial</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>25000-23-42-000-2016-02740-01</t>
+          <t>11001-11-02-000-2019-07466-01</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>31-10-2024</t>
+          <t>25-10-2024</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>TA Cundinamarca – Rad. 25000-23-42-000-2016-02740-01 – Nulidad y restablecimiento sancion disciplinaria policial culpa grave frente a dolo</t>
+          <t>CNDJ – Rad. 11001-11-02-000-2019-07466-01 – Exclusion de la profesion por ejercer estando suspendido</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>apreciación probatoria; sana crítica; valoración probatoria</t>
+          <t>apreciación probatoria</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1_1OrQcyc38GEWJits46ul3-95g66AeIo/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1T4ZizI1hcgg2OI4GpHy67qErDEC6_kGh/view?usp=drivesdk</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>1_1OrQcyc38GEWJits46ul3-95g66AeIo</t>
+          <t>1T4ZizI1hcgg2OI4GpHy67qErDEC6_kGh</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí – término ausente</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>El texto no contiene ninguno de los términos buscados; el hit del índice de Drive fue un falso positivo.</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Confirma la sentencia de primera instancia (exclusión del abogado).</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>ninguno de los 6 términos aparece en el texto</t>
         </is>
       </c>
     </row>
@@ -1325,6 +1487,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1377,6 +1541,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1429,6 +1595,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1481,6 +1649,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1533,6 +1703,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K21" s="2" t="n"/>
+      <c r="L21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1585,6 +1757,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1637,6 +1811,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K23" s="2" t="n"/>
+      <c r="L23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1689,6 +1865,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K24" s="2" t="n"/>
+      <c r="L24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1741,6 +1919,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K25" s="2" t="n"/>
+      <c r="L25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1793,6 +1973,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K26" s="2" t="n"/>
+      <c r="L26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1845,6 +2027,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K27" s="2" t="n"/>
+      <c r="L27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1897,6 +2081,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K28" s="2" t="n"/>
+      <c r="L28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1949,6 +2135,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K29" s="2" t="n"/>
+      <c r="L29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2001,6 +2189,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K30" s="2" t="n"/>
+      <c r="L30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2053,6 +2243,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K31" s="2" t="n"/>
+      <c r="L31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2105,6 +2297,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K32" s="2" t="n"/>
+      <c r="L32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2157,6 +2351,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K33" s="2" t="n"/>
+      <c r="L33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2209,6 +2405,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K34" s="2" t="n"/>
+      <c r="L34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2226,7 +2424,7 @@
           <t>11001-03-25-000-2011-00207-00</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="inlineStr">
         <is>
           <t>CE Secc. 2ª – Rad. 11001-03-25-000-2011-00207-00 (0722-11)</t>
@@ -2257,6 +2455,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K35" s="2" t="n"/>
+      <c r="L35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2274,7 +2474,7 @@
           <t>0051-2013</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="inlineStr">
         <is>
           <t>CE Secc. 2ª – Rad. 0051-2013</t>
@@ -2305,6 +2505,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K36" s="2" t="n"/>
+      <c r="L36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2357,6 +2559,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K37" s="2" t="n"/>
+      <c r="L37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2409,6 +2613,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K38" s="2" t="n"/>
+      <c r="L38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2461,6 +2667,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K39" s="2" t="n"/>
+      <c r="L39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2513,6 +2721,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K40" s="2" t="n"/>
+      <c r="L40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2565,6 +2775,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K41" s="2" t="n"/>
+      <c r="L41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2617,6 +2829,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K42" s="2" t="n"/>
+      <c r="L42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2669,6 +2883,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K43" s="2" t="n"/>
+      <c r="L43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2721,6 +2937,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K44" s="2" t="n"/>
+      <c r="L44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2773,6 +2991,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K45" s="2" t="n"/>
+      <c r="L45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2825,6 +3045,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K46" s="2" t="n"/>
+      <c r="L46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2877,6 +3099,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K47" s="2" t="n"/>
+      <c r="L47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2929,6 +3153,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K48" s="2" t="n"/>
+      <c r="L48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2981,6 +3207,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K49" s="2" t="n"/>
+      <c r="L49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3033,6 +3261,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K50" s="2" t="n"/>
+      <c r="L50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3085,6 +3315,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K51" s="2" t="n"/>
+      <c r="L51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3137,6 +3369,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K52" s="2" t="n"/>
+      <c r="L52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3189,6 +3423,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K53" s="2" t="n"/>
+      <c r="L53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3241,6 +3477,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K54" s="2" t="n"/>
+      <c r="L54" s="2" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3293,6 +3531,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K55" s="2" t="n"/>
+      <c r="L55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3345,6 +3585,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K56" s="2" t="n"/>
+      <c r="L56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3397,6 +3639,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K57" s="2" t="n"/>
+      <c r="L57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3449,6 +3693,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K58" s="2" t="n"/>
+      <c r="L58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3501,6 +3747,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K59" s="2" t="n"/>
+      <c r="L59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3553,6 +3801,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K60" s="2" t="n"/>
+      <c r="L60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3605,6 +3855,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K61" s="2" t="n"/>
+      <c r="L61" s="2" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3657,6 +3909,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K62" s="2" t="n"/>
+      <c r="L62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3709,6 +3963,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K63" s="2" t="n"/>
+      <c r="L63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3761,6 +4017,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K64" s="2" t="n"/>
+      <c r="L64" s="2" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3813,6 +4071,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K65" s="2" t="n"/>
+      <c r="L65" s="2" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3865,6 +4125,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K66" s="2" t="n"/>
+      <c r="L66" s="2" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -3917,6 +4179,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K67" s="2" t="n"/>
+      <c r="L67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3969,6 +4233,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K68" s="2" t="n"/>
+      <c r="L68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4021,6 +4287,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K69" s="2" t="n"/>
+      <c r="L69" s="2" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4073,6 +4341,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K70" s="2" t="n"/>
+      <c r="L70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4125,6 +4395,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K71" s="2" t="n"/>
+      <c r="L71" s="2" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4177,6 +4449,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K72" s="2" t="n"/>
+      <c r="L72" s="2" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4229,6 +4503,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K73" s="2" t="n"/>
+      <c r="L73" s="2" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4281,6 +4557,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K74" s="2" t="n"/>
+      <c r="L74" s="2" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4333,6 +4611,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K75" s="2" t="n"/>
+      <c r="L75" s="2" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4385,6 +4665,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K76" s="2" t="n"/>
+      <c r="L76" s="2" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -4437,6 +4719,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K77" s="2" t="n"/>
+      <c r="L77" s="2" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4489,6 +4773,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K78" s="2" t="n"/>
+      <c r="L78" s="2" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -4541,6 +4827,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K79" s="2" t="n"/>
+      <c r="L79" s="2" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -4593,6 +4881,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K80" s="2" t="n"/>
+      <c r="L80" s="2" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -4645,6 +4935,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K81" s="2" t="n"/>
+      <c r="L81" s="2" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -4697,6 +4989,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K82" s="2" t="n"/>
+      <c r="L82" s="2" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -4749,6 +5043,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K83" s="2" t="n"/>
+      <c r="L83" s="2" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -4801,6 +5097,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K84" s="2" t="n"/>
+      <c r="L84" s="2" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -4853,6 +5151,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K85" s="2" t="n"/>
+      <c r="L85" s="2" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -4905,6 +5205,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K86" s="2" t="n"/>
+      <c r="L86" s="2" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -4957,6 +5259,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K87" s="2" t="n"/>
+      <c r="L87" s="2" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5009,6 +5313,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K88" s="2" t="n"/>
+      <c r="L88" s="2" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -5061,6 +5367,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K89" s="2" t="n"/>
+      <c r="L89" s="2" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -5113,6 +5421,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K90" s="2" t="n"/>
+      <c r="L90" s="2" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -5165,6 +5475,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K91" s="2" t="n"/>
+      <c r="L91" s="2" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -5217,6 +5529,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K92" s="2" t="n"/>
+      <c r="L92" s="2" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -5269,6 +5583,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K93" s="2" t="n"/>
+      <c r="L93" s="2" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -5321,6 +5637,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K94" s="2" t="n"/>
+      <c r="L94" s="2" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -5373,6 +5691,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K95" s="2" t="n"/>
+      <c r="L95" s="2" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -5425,6 +5745,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K96" s="2" t="n"/>
+      <c r="L96" s="2" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -5477,6 +5799,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K97" s="2" t="n"/>
+      <c r="L97" s="2" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -5529,6 +5853,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K98" s="2" t="n"/>
+      <c r="L98" s="2" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -5581,6 +5907,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K99" s="2" t="n"/>
+      <c r="L99" s="2" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -5633,6 +5961,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K100" s="2" t="n"/>
+      <c r="L100" s="2" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -5685,6 +6015,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K101" s="2" t="n"/>
+      <c r="L101" s="2" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -5737,6 +6069,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K102" s="2" t="n"/>
+      <c r="L102" s="2" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -5789,6 +6123,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K103" s="2" t="n"/>
+      <c r="L103" s="2" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -5841,6 +6177,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K104" s="2" t="n"/>
+      <c r="L104" s="2" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -5893,6 +6231,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K105" s="2" t="n"/>
+      <c r="L105" s="2" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -5945,6 +6285,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K106" s="2" t="n"/>
+      <c r="L106" s="2" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -5997,6 +6339,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K107" s="2" t="n"/>
+      <c r="L107" s="2" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -6049,6 +6393,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K108" s="2" t="n"/>
+      <c r="L108" s="2" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -6101,6 +6447,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K109" s="2" t="n"/>
+      <c r="L109" s="2" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -6153,6 +6501,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K110" s="2" t="n"/>
+      <c r="L110" s="2" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -6205,6 +6555,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K111" s="2" t="n"/>
+      <c r="L111" s="2" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -6257,6 +6609,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K112" s="2" t="n"/>
+      <c r="L112" s="2" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -6309,6 +6663,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K113" s="2" t="n"/>
+      <c r="L113" s="2" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -6361,6 +6717,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K114" s="2" t="n"/>
+      <c r="L114" s="2" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -6413,6 +6771,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K115" s="2" t="n"/>
+      <c r="L115" s="2" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -6465,6 +6825,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K116" s="2" t="n"/>
+      <c r="L116" s="2" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -6517,6 +6879,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K117" s="2" t="n"/>
+      <c r="L117" s="2" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -6569,6 +6933,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K118" s="2" t="n"/>
+      <c r="L118" s="2" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -6621,6 +6987,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K119" s="2" t="n"/>
+      <c r="L119" s="2" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -6673,6 +7041,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K120" s="2" t="n"/>
+      <c r="L120" s="2" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -6725,6 +7095,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K121" s="2" t="n"/>
+      <c r="L121" s="2" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -6777,6 +7149,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K122" s="2" t="n"/>
+      <c r="L122" s="2" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -6829,6 +7203,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K123" s="2" t="n"/>
+      <c r="L123" s="2" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -6881,6 +7257,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K124" s="2" t="n"/>
+      <c r="L124" s="2" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -6933,6 +7311,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K125" s="2" t="n"/>
+      <c r="L125" s="2" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -6985,6 +7365,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K126" s="2" t="n"/>
+      <c r="L126" s="2" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -7037,6 +7419,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K127" s="2" t="n"/>
+      <c r="L127" s="2" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -7089,6 +7473,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K128" s="2" t="n"/>
+      <c r="L128" s="2" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -7141,6 +7527,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K129" s="2" t="n"/>
+      <c r="L129" s="2" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -7193,6 +7581,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K130" s="2" t="n"/>
+      <c r="L130" s="2" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -7245,6 +7635,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K131" s="2" t="n"/>
+      <c r="L131" s="2" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -7297,6 +7689,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K132" s="2" t="n"/>
+      <c r="L132" s="2" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -7349,6 +7743,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K133" s="2" t="n"/>
+      <c r="L133" s="2" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -7401,6 +7797,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K134" s="2" t="n"/>
+      <c r="L134" s="2" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -7453,6 +7851,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K135" s="2" t="n"/>
+      <c r="L135" s="2" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -7505,6 +7905,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K136" s="2" t="n"/>
+      <c r="L136" s="2" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -7557,6 +7959,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K137" s="2" t="n"/>
+      <c r="L137" s="2" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -7609,6 +8013,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K138" s="2" t="n"/>
+      <c r="L138" s="2" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -7661,6 +8067,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K139" s="2" t="n"/>
+      <c r="L139" s="2" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -7713,6 +8121,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K140" s="2" t="n"/>
+      <c r="L140" s="2" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -7765,6 +8175,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K141" s="2" t="n"/>
+      <c r="L141" s="2" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -7777,8 +8189,8 @@
           <t>Corte Constitucional</t>
         </is>
       </c>
-      <c r="C142" s="2" t="inlineStr"/>
-      <c r="D142" s="2" t="inlineStr"/>
+      <c r="C142" s="2" t="n"/>
+      <c r="D142" s="2" t="n"/>
       <c r="E142" s="2" t="inlineStr">
         <is>
           <t>CC – Sent. SU-901 de 2005</t>
@@ -7809,6 +8221,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K142" s="2" t="n"/>
+      <c r="L142" s="2" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -7821,8 +8235,8 @@
           <t>Corte Constitucional</t>
         </is>
       </c>
-      <c r="C143" s="2" t="inlineStr"/>
-      <c r="D143" s="2" t="inlineStr"/>
+      <c r="C143" s="2" t="n"/>
+      <c r="D143" s="2" t="n"/>
       <c r="E143" s="2" t="inlineStr">
         <is>
           <t>CC – Sent. T-235 de 2025</t>
@@ -7853,6 +8267,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K143" s="2" t="n"/>
+      <c r="L143" s="2" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -7905,6 +8321,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K144" s="2" t="n"/>
+      <c r="L144" s="2" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -7922,7 +8340,7 @@
           <t>IUS E-2014-239195 IUC D-2015-701369</t>
         </is>
       </c>
-      <c r="D145" s="2" t="inlineStr"/>
+      <c r="D145" s="2" t="n"/>
       <c r="E145" s="2" t="inlineStr">
         <is>
           <t>Otros – PGN Delegada Vigilancia Admtiva – Rad. IUS E-2014-239195 IUC D-2015-701369 – Sancion destitucion docente abuso sexual menor</t>
@@ -7953,6 +8371,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K145" s="2" t="n"/>
+      <c r="L145" s="2" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -8005,6 +8425,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K146" s="2" t="n"/>
+      <c r="L146" s="2" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -8057,6 +8479,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K147" s="2" t="n"/>
+      <c r="L147" s="2" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -8109,6 +8533,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K148" s="2" t="n"/>
+      <c r="L148" s="2" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -8161,6 +8587,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K149" s="2" t="n"/>
+      <c r="L149" s="2" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -8213,6 +8641,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K150" s="2" t="n"/>
+      <c r="L150" s="2" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -8265,6 +8695,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K151" s="2" t="n"/>
+      <c r="L151" s="2" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -8317,6 +8749,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K152" s="2" t="n"/>
+      <c r="L152" s="2" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -8369,6 +8803,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K153" s="2" t="n"/>
+      <c r="L153" s="2" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -8421,6 +8857,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K154" s="2" t="n"/>
+      <c r="L154" s="2" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -8473,6 +8911,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K155" s="2" t="n"/>
+      <c r="L155" s="2" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -8525,6 +8965,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K156" s="2" t="n"/>
+      <c r="L156" s="2" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -8577,6 +9019,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K157" s="2" t="n"/>
+      <c r="L157" s="2" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -8594,7 +9038,7 @@
           <t>2017-05284</t>
         </is>
       </c>
-      <c r="D158" s="2" t="inlineStr"/>
+      <c r="D158" s="2" t="n"/>
       <c r="E158" s="2" t="inlineStr">
         <is>
           <t>CE Secc. 2ª – Rad. 2017-05284 – Derechos políticos concejal terminado período</t>
@@ -8625,6 +9069,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K158" s="2" t="n"/>
+      <c r="L158" s="2" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -8637,8 +9083,8 @@
           <t>Consejo de Estado – Sec. 2ª</t>
         </is>
       </c>
-      <c r="C159" s="2" t="inlineStr"/>
-      <c r="D159" s="2" t="inlineStr"/>
+      <c r="C159" s="2" t="n"/>
+      <c r="D159" s="2" t="n"/>
       <c r="E159" s="2" t="inlineStr">
         <is>
           <t>CE Secc. 2ª – Rad. 11001-03-25-000-2011-00574-00(2201-11)</t>
@@ -8669,6 +9115,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K159" s="2" t="n"/>
+      <c r="L159" s="2" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -8681,8 +9129,8 @@
           <t>Consejo de Estado – Sec. 2ª</t>
         </is>
       </c>
-      <c r="C160" s="2" t="inlineStr"/>
-      <c r="D160" s="2" t="inlineStr"/>
+      <c r="C160" s="2" t="n"/>
+      <c r="D160" s="2" t="n"/>
       <c r="E160" s="2" t="inlineStr">
         <is>
           <t>CE Secc. 2ª – Rad. 11001-03-25-000-2011-00207-00(0722-11)</t>
@@ -8713,6 +9161,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K160" s="2" t="n"/>
+      <c r="L160" s="2" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -8730,7 +9180,7 @@
           <t>6432-2018</t>
         </is>
       </c>
-      <c r="D161" s="2" t="inlineStr"/>
+      <c r="D161" s="2" t="n"/>
       <c r="E161" s="2" t="inlineStr">
         <is>
           <t>CE Secc. 2ª – Rad. 6432-2018 – Laboral administrativo</t>
@@ -8761,6 +9211,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K161" s="2" t="n"/>
+      <c r="L161" s="2" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -8813,6 +9265,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K162" s="2" t="n"/>
+      <c r="L162" s="2" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -8865,6 +9319,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K163" s="2" t="n"/>
+      <c r="L163" s="2" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -8917,6 +9373,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K164" s="2" t="n"/>
+      <c r="L164" s="2" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -8969,6 +9427,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K165" s="2" t="n"/>
+      <c r="L165" s="2" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -9021,6 +9481,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K166" s="2" t="n"/>
+      <c r="L166" s="2" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -9073,6 +9535,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K167" s="2" t="n"/>
+      <c r="L167" s="2" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -9125,6 +9589,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K168" s="2" t="n"/>
+      <c r="L168" s="2" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -9177,6 +9643,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K169" s="2" t="n"/>
+      <c r="L169" s="2" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -9229,6 +9697,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K170" s="2" t="n"/>
+      <c r="L170" s="2" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -9281,6 +9751,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K171" s="2" t="n"/>
+      <c r="L171" s="2" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -9333,6 +9805,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K172" s="2" t="n"/>
+      <c r="L172" s="2" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -9385,6 +9859,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K173" s="2" t="n"/>
+      <c r="L173" s="2" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -9437,6 +9913,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K174" s="2" t="n"/>
+      <c r="L174" s="2" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -9489,6 +9967,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K175" s="2" t="n"/>
+      <c r="L175" s="2" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -9541,6 +10021,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K176" s="2" t="n"/>
+      <c r="L176" s="2" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
@@ -9593,6 +10075,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K177" s="2" t="n"/>
+      <c r="L177" s="2" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -9645,6 +10129,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K178" s="2" t="n"/>
+      <c r="L178" s="2" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -9697,6 +10183,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K179" s="2" t="n"/>
+      <c r="L179" s="2" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -9749,6 +10237,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K180" s="2" t="n"/>
+      <c r="L180" s="2" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -9801,6 +10291,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K181" s="2" t="n"/>
+      <c r="L181" s="2" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -9818,7 +10310,7 @@
           <t>469-24</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr"/>
+      <c r="D182" s="2" t="n"/>
       <c r="E182" s="2" t="inlineStr">
         <is>
           <t>CE Secc. 3ª – Rad. 469-24 – Reparación directa</t>
@@ -9849,6 +10341,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K182" s="2" t="n"/>
+      <c r="L182" s="2" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -9866,7 +10360,7 @@
           <t>38806</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr"/>
+      <c r="D183" s="2" t="n"/>
       <c r="E183" s="2" t="inlineStr">
         <is>
           <t>CE Secc. 3ª – Rad. 38806 – Reparación directa, muerte menor intoxicación gas</t>
@@ -9897,6 +10391,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K183" s="2" t="n"/>
+      <c r="L183" s="2" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -9949,6 +10445,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K184" s="2" t="n"/>
+      <c r="L184" s="2" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
@@ -10001,6 +10499,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K185" s="2" t="n"/>
+      <c r="L185" s="2" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -10053,6 +10553,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K186" s="2" t="n"/>
+      <c r="L186" s="2" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
@@ -10105,6 +10607,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K187" s="2" t="n"/>
+      <c r="L187" s="2" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -10157,6 +10661,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K188" s="2" t="n"/>
+      <c r="L188" s="2" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
@@ -10209,6 +10715,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K189" s="2" t="n"/>
+      <c r="L189" s="2" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -10261,6 +10769,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K190" s="2" t="n"/>
+      <c r="L190" s="2" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
@@ -10313,6 +10823,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K191" s="2" t="n"/>
+      <c r="L191" s="2" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -10365,6 +10877,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K192" s="2" t="n"/>
+      <c r="L192" s="2" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -10417,6 +10931,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K193" s="2" t="n"/>
+      <c r="L193" s="2" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -10469,6 +10985,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K194" s="2" t="n"/>
+      <c r="L194" s="2" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -10521,6 +11039,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K195" s="2" t="n"/>
+      <c r="L195" s="2" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -10573,6 +11093,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K196" s="2" t="n"/>
+      <c r="L196" s="2" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
@@ -10625,6 +11147,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K197" s="2" t="n"/>
+      <c r="L197" s="2" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -10677,6 +11201,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K198" s="2" t="n"/>
+      <c r="L198" s="2" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
@@ -10729,6 +11255,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K199" s="2" t="n"/>
+      <c r="L199" s="2" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -10781,6 +11309,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K200" s="2" t="n"/>
+      <c r="L200" s="2" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
@@ -10833,6 +11363,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K201" s="2" t="n"/>
+      <c r="L201" s="2" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -10885,6 +11417,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K202" s="2" t="n"/>
+      <c r="L202" s="2" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
@@ -10937,6 +11471,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K203" s="2" t="n"/>
+      <c r="L203" s="2" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -10989,6 +11525,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K204" s="2" t="n"/>
+      <c r="L204" s="2" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
@@ -11041,6 +11579,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K205" s="2" t="n"/>
+      <c r="L205" s="2" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -11093,6 +11633,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K206" s="2" t="n"/>
+      <c r="L206" s="2" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
@@ -11145,6 +11687,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K207" s="2" t="n"/>
+      <c r="L207" s="2" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -11197,6 +11741,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K208" s="2" t="n"/>
+      <c r="L208" s="2" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
@@ -11249,6 +11795,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K209" s="2" t="n"/>
+      <c r="L209" s="2" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -11301,6 +11849,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K210" s="2" t="n"/>
+      <c r="L210" s="2" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
@@ -11353,6 +11903,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K211" s="2" t="n"/>
+      <c r="L211" s="2" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
@@ -11405,6 +11957,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K212" s="2" t="n"/>
+      <c r="L212" s="2" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
@@ -11457,6 +12011,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K213" s="2" t="n"/>
+      <c r="L213" s="2" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
@@ -11509,6 +12065,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K214" s="2" t="n"/>
+      <c r="L214" s="2" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
@@ -11561,6 +12119,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K215" s="2" t="n"/>
+      <c r="L215" s="2" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
@@ -11613,6 +12173,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K216" s="2" t="n"/>
+      <c r="L216" s="2" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
@@ -11665,6 +12227,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K217" s="2" t="n"/>
+      <c r="L217" s="2" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
@@ -11717,6 +12281,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K218" s="2" t="n"/>
+      <c r="L218" s="2" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
@@ -11769,6 +12335,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K219" s="2" t="n"/>
+      <c r="L219" s="2" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -11821,6 +12389,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K220" s="2" t="n"/>
+      <c r="L220" s="2" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
@@ -11873,6 +12443,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K221" s="2" t="n"/>
+      <c r="L221" s="2" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
@@ -11925,6 +12497,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K222" s="2" t="n"/>
+      <c r="L222" s="2" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
@@ -11977,6 +12551,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K223" s="2" t="n"/>
+      <c r="L223" s="2" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
@@ -12029,6 +12605,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K224" s="2" t="n"/>
+      <c r="L224" s="2" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
@@ -12081,6 +12659,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K225" s="2" t="n"/>
+      <c r="L225" s="2" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
@@ -12093,7 +12673,7 @@
           <t>Corte Constitucional</t>
         </is>
       </c>
-      <c r="C226" s="2" t="inlineStr"/>
+      <c r="C226" s="2" t="n"/>
       <c r="D226" s="2" t="inlineStr">
         <is>
           <t>18-12-2023</t>
@@ -12129,6 +12709,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K226" s="2" t="n"/>
+      <c r="L226" s="2" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
@@ -12181,6 +12763,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K227" s="2" t="n"/>
+      <c r="L227" s="2" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
@@ -12233,6 +12817,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K228" s="2" t="n"/>
+      <c r="L228" s="2" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
@@ -12285,6 +12871,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K229" s="2" t="n"/>
+      <c r="L229" s="2" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
@@ -12337,6 +12925,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K230" s="2" t="n"/>
+      <c r="L230" s="2" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
@@ -12389,6 +12979,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K231" s="2" t="n"/>
+      <c r="L231" s="2" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
@@ -12441,6 +13033,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K232" s="2" t="n"/>
+      <c r="L232" s="2" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
@@ -12453,7 +13047,7 @@
           <t>Corte Constitucional</t>
         </is>
       </c>
-      <c r="C233" s="2" t="inlineStr"/>
+      <c r="C233" s="2" t="n"/>
       <c r="D233" s="2" t="inlineStr">
         <is>
           <t>17-03-2025</t>
@@ -12489,6 +13083,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K233" s="2" t="n"/>
+      <c r="L233" s="2" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
@@ -12541,6 +13137,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K234" s="2" t="n"/>
+      <c r="L234" s="2" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
@@ -12553,7 +13151,7 @@
           <t>Corte Constitucional</t>
         </is>
       </c>
-      <c r="C235" s="2" t="inlineStr"/>
+      <c r="C235" s="2" t="n"/>
       <c r="D235" s="2" t="inlineStr">
         <is>
           <t>08-05-2025</t>
@@ -12589,6 +13187,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K235" s="2" t="n"/>
+      <c r="L235" s="2" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
@@ -12641,6 +13241,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K236" s="2" t="n"/>
+      <c r="L236" s="2" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
@@ -12653,8 +13255,8 @@
           <t>Corte Suprema de Justicia</t>
         </is>
       </c>
-      <c r="C237" s="2" t="inlineStr"/>
-      <c r="D237" s="2" t="inlineStr"/>
+      <c r="C237" s="2" t="n"/>
+      <c r="D237" s="2" t="n"/>
       <c r="E237" s="2" t="inlineStr">
         <is>
           <t>CSJ Penal – AP2765-2025 (68644)</t>
@@ -12685,6 +13287,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K237" s="2" t="n"/>
+      <c r="L237" s="2" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
@@ -12697,8 +13301,8 @@
           <t>Corte Suprema de Justicia</t>
         </is>
       </c>
-      <c r="C238" s="2" t="inlineStr"/>
-      <c r="D238" s="2" t="inlineStr"/>
+      <c r="C238" s="2" t="n"/>
+      <c r="D238" s="2" t="n"/>
       <c r="E238" s="2" t="inlineStr">
         <is>
           <t>CSJ Penal – SP1775-2025 (60554)</t>
@@ -12729,6 +13333,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K238" s="2" t="n"/>
+      <c r="L238" s="2" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
@@ -12741,8 +13347,8 @@
           <t>Corte Suprema de Justicia</t>
         </is>
       </c>
-      <c r="C239" s="2" t="inlineStr"/>
-      <c r="D239" s="2" t="inlineStr"/>
+      <c r="C239" s="2" t="n"/>
+      <c r="D239" s="2" t="n"/>
       <c r="E239" s="2" t="inlineStr">
         <is>
           <t>CSJ Penal – SP1606-2025 (63257)</t>
@@ -12773,6 +13379,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K239" s="2" t="n"/>
+      <c r="L239" s="2" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
@@ -12785,8 +13393,8 @@
           <t>Corte Suprema de Justicia</t>
         </is>
       </c>
-      <c r="C240" s="2" t="inlineStr"/>
-      <c r="D240" s="2" t="inlineStr"/>
+      <c r="C240" s="2" t="n"/>
+      <c r="D240" s="2" t="n"/>
       <c r="E240" s="2" t="inlineStr">
         <is>
           <t>CSJ Penal – SP2487-2024 (57115)</t>
@@ -12817,6 +13425,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K240" s="2" t="n"/>
+      <c r="L240" s="2" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
@@ -12869,6 +13479,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K241" s="2" t="n"/>
+      <c r="L241" s="2" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
@@ -12921,6 +13533,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K242" s="2" t="n"/>
+      <c r="L242" s="2" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
@@ -12973,6 +13587,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K243" s="2" t="n"/>
+      <c r="L243" s="2" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
@@ -13025,6 +13641,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K244" s="2" t="n"/>
+      <c r="L244" s="2" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
@@ -13077,6 +13695,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K245" s="2" t="n"/>
+      <c r="L245" s="2" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
@@ -13129,6 +13749,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K246" s="2" t="n"/>
+      <c r="L246" s="2" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
@@ -13181,6 +13803,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K247" s="2" t="n"/>
+      <c r="L247" s="2" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
@@ -13233,6 +13857,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K248" s="2" t="n"/>
+      <c r="L248" s="2" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
@@ -13285,6 +13911,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K249" s="2" t="n"/>
+      <c r="L249" s="2" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
@@ -13337,6 +13965,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K250" s="2" t="n"/>
+      <c r="L250" s="2" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
@@ -13389,6 +14019,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K251" s="2" t="n"/>
+      <c r="L251" s="2" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
@@ -13401,7 +14033,7 @@
           <t>Juzgado</t>
         </is>
       </c>
-      <c r="C252" s="2" t="inlineStr"/>
+      <c r="C252" s="2" t="n"/>
       <c r="D252" s="2" t="inlineStr">
         <is>
           <t>01-08-2025</t>
@@ -13437,6 +14069,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K252" s="2" t="n"/>
+      <c r="L252" s="2" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
@@ -13449,8 +14083,8 @@
           <t>Otros</t>
         </is>
       </c>
-      <c r="C253" s="2" t="inlineStr"/>
-      <c r="D253" s="2" t="inlineStr"/>
+      <c r="C253" s="2" t="n"/>
+      <c r="D253" s="2" t="n"/>
       <c r="E253" s="2" t="inlineStr">
         <is>
           <t>Otros – Libro Los hechos en la sentencia penal</t>
@@ -13481,6 +14115,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K253" s="2" t="n"/>
+      <c r="L253" s="2" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
@@ -13533,6 +14169,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K254" s="2" t="n"/>
+      <c r="L254" s="2" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
@@ -13585,6 +14223,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K255" s="2" t="n"/>
+      <c r="L255" s="2" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
@@ -13637,6 +14277,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K256" s="2" t="n"/>
+      <c r="L256" s="2" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
@@ -13689,6 +14331,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K257" s="2" t="n"/>
+      <c r="L257" s="2" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
@@ -13741,6 +14385,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K258" s="2" t="n"/>
+      <c r="L258" s="2" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
@@ -13793,6 +14439,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K259" s="2" t="n"/>
+      <c r="L259" s="2" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
@@ -13845,9 +14493,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="K260" s="2" t="n"/>
+      <c r="L260" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J260"/>
+  <autoFilter ref="A1:L260"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13858,7 +14508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -13881,21 +14531,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LIMITACIÓN: el buscador de Drive no garantiza que el término aparezca en la providencia; no se leyó el contenido. La columna «Verificado en texto» está en No para todas.</t>
+          <t>Nivel A1: leída y central para valoración probatoria disciplinaria (9). Nivel A2: leída; el tema probatorio es tangencial (5). Nivel D: leída; falso positivo (1).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Nivel A: el título de la providencia señala tema probatorio y disciplinario. Nivel B: disciplinaria, coincidencia solo de índice. Nivel C: otras materias (fiscal, contractual, laboral, etc.).</t>
+          <t>Nivel B (disciplinaria) y C (otras materias): NO leídas; solo coincidencia de índice del buscador de Drive, que no garantiza que el término aparezca. Verificado en texto = «No».</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Antes de citar cualquier providencia, leer el texto y extraer la regla con cita textual.</t>
+          <t>Las citas textuales de las filas A1/A2 provienen de la lectura de la providencia; los números de párrafo se indican solo cuando constan en el texto. Verificar contra el original antes de citar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Los fallos 0086-2014 y CNDJ 2021-00235-02 se leyeron completos; el resto mediante lectura dirigida (búsqueda de términos, problema jurídico, regla y decisión), no integral.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar esquema de reglas por tema y auditoría de radicados en la matriz
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HFz41Xq5pxE4jPsKEtG9Mg
</commit_message>
<xml_diff>
--- a/Matriz_Valoracion_Probatoria_Disciplinaria.xlsx
+++ b/Matriz_Valoracion_Probatoria_Disciplinaria.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L260"/>
+  <dimension ref="A1:M260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -446,6 +446,7 @@
     <col width="90" customWidth="1" min="10" max="10"/>
     <col width="50" customWidth="1" min="11" max="11"/>
     <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="46" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -509,6 +510,11 @@
           <t>Términos hallados en el texto (n.º de apariciones)</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Verificación del radicado (título de Drive vs. texto)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -571,6 +577,11 @@
           <t>prueba indiciaria / indicios (3)</t>
         </is>
       </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -633,6 +644,11 @@
           <t>sana crítica (2); referencias a prueba lícita/ilícita de mensajes de voz (lectura completa)</t>
         </is>
       </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -695,6 +711,11 @@
           <t>valoración probatoria (2), indicios (3)</t>
         </is>
       </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el texto completo (leído)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -757,6 +778,11 @@
           <t>prueba ilícita / exclusión (16), valoración probatoria (5), apreciación probatoria (1)</t>
         </is>
       </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el texto completo (leído)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -819,6 +845,11 @@
           <t>indicios (20), sana crítica (4), valoración probatoria (5), prueba ilícita (1)</t>
         </is>
       </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -881,6 +912,11 @@
           <t>sana crítica (3), prueba trasladada (1)</t>
         </is>
       </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -943,6 +979,11 @@
           <t>valoración probatoria (1), sana crítica (2), prueba ilícita (1), indicios (1)</t>
         </is>
       </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1005,6 +1046,11 @@
           <t>prueba trasladada, sana crítica, valoración probatoria (lectura completa)</t>
         </is>
       </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1063,6 +1109,11 @@
           <t>valoración probatoria (4), sana crítica (2)</t>
         </is>
       </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Título sin radicado completo; no comparable</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1125,6 +1176,11 @@
           <t>valoración probatoria (1), sana crítica (2), indicios (1)</t>
         </is>
       </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el texto completo (leído)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1187,6 +1243,11 @@
           <t>valoración probatoria (2), indicios (12; uso no verificado)</t>
         </is>
       </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el texto completo (leído)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1249,6 +1310,11 @@
           <t>prueba trasladada (5), valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1311,6 +1377,11 @@
           <t>prueba trasladada (cita de doctrina de la Sala), valoración</t>
         </is>
       </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Título sin radicado completo; no comparable</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1373,6 +1444,11 @@
           <t>valoración probatoria (2), sana crítica (2)</t>
         </is>
       </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1435,6 +1511,11 @@
           <t>valoración probatoria (2)</t>
         </is>
       </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1497,6 +1578,11 @@
           <t>valoración probatoria (2); sana crítica (6); indicios/prueba indiciaria (4)</t>
         </is>
       </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1559,6 +1645,11 @@
           <t>prueba ilícita/exclusión (9)</t>
         </is>
       </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1617,6 +1708,11 @@
           <t>valoración probatoria (4); apreciación probatoria (1); sana crítica (7); prueba trasladada (2)</t>
         </is>
       </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>DESAJUSTE confirmado: el archivo contiene la sentencia 76001-23-33-000-2012-00394-01 (0941-19, Ecopetrol, 28-01-2021), no la 0722-11. Duplicado de otra fila.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1675,6 +1771,11 @@
           <t>valoración probatoria (3); apreciación probatoria (3); sana crítica (2)</t>
         </is>
       </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1737,6 +1838,11 @@
           <t>sana crítica (3)</t>
         </is>
       </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1799,6 +1905,11 @@
           <t>valoración probatoria (7); sana crítica (3)</t>
         </is>
       </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>DESAJUSTE confirmado: el archivo contiene la sentencia 15001-23-33-000-2015-00336-01 (1286-2021, DIH, 13-04-2023), no la 0058-12. Duplicado de otra fila.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1861,6 +1972,11 @@
           <t>valoración probatoria (8); sana crítica (5)</t>
         </is>
       </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>DESAJUSTE confirmado: el archivo contiene la sentencia 05001-23-33-000-2016-02320-01 (3358-2022, dádivas, 11-05-2023), no la 1566-12. Duplicado de otra fila.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1923,6 +2039,11 @@
           <t>valoración probatoria (6); sana crítica (3)</t>
         </is>
       </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1985,6 +2106,11 @@
           <t>valoración probatoria (6); sana crítica (8)</t>
         </is>
       </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2047,6 +2173,11 @@
           <t>valoración probatoria (2); prueba ilícita/exclusión (1)</t>
         </is>
       </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2109,6 +2240,11 @@
           <t>valoración probatoria (3); sana crítica (2)</t>
         </is>
       </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2171,6 +2307,11 @@
           <t>valoración probatoria (2); sana crítica (7)</t>
         </is>
       </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2233,6 +2374,11 @@
           <t>valoración probatoria (1); sana crítica (3)</t>
         </is>
       </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2295,6 +2441,11 @@
           <t>valoración probatoria (2); apreciación probatoria (1); sana crítica (8)</t>
         </is>
       </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2357,6 +2508,11 @@
           <t>valoración probatoria (19); sana crítica (7)</t>
         </is>
       </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2419,6 +2575,11 @@
           <t>valoración probatoria (8); sana crítica (11)</t>
         </is>
       </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2481,6 +2642,11 @@
           <t>valoración probatoria (8); sana crítica (9); indicios/prueba indiciaria (1)</t>
         </is>
       </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>Título sin radicado completo; no comparable</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2543,6 +2709,11 @@
           <t>valoración probatoria (8); sana crítica (9); indicios/prueba indiciaria (1)</t>
         </is>
       </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2605,6 +2776,11 @@
           <t>valoración probatoria (2); sana crítica (5); indicios/prueba indiciaria (4)</t>
         </is>
       </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2667,6 +2843,11 @@
           <t>valoración probatoria (4); apreciación probatoria (3); sana crítica (2)</t>
         </is>
       </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2729,6 +2910,11 @@
           <t>valoración probatoria (8); sana crítica (5)</t>
         </is>
       </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2791,6 +2977,11 @@
           <t>valoración probatoria (4); sana crítica (4); indicios/prueba indiciaria (17); prueba trasladada (1)</t>
         </is>
       </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2853,6 +3044,11 @@
           <t>valoración probatoria (2); sana crítica (2); indicios/prueba indiciaria (2)</t>
         </is>
       </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2915,6 +3111,11 @@
           <t>valoración probatoria (7); sana crítica (7); indicios/prueba indiciaria (5); prueba trasladada (6)</t>
         </is>
       </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2977,6 +3178,11 @@
           <t>valoración probatoria (4); sana crítica (6); indicios/prueba indiciaria (4); prueba trasladada (6)</t>
         </is>
       </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3039,6 +3245,11 @@
           <t>valoración probatoria (2); sana crítica (5); indicios/prueba indiciaria (1)</t>
         </is>
       </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3101,6 +3312,11 @@
           <t>sana crítica (2)</t>
         </is>
       </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3163,6 +3379,11 @@
           <t>valoración probatoria (2); sana crítica (3)</t>
         </is>
       </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3225,6 +3446,11 @@
           <t>valoración probatoria (5); sana crítica (8)</t>
         </is>
       </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3287,6 +3513,11 @@
           <t>valoración probatoria (3); sana crítica (3)</t>
         </is>
       </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3349,6 +3580,11 @@
           <t>valoración probatoria (1); sana crítica (3)</t>
         </is>
       </c>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3411,6 +3647,11 @@
           <t>valoración probatoria (3); apreciación probatoria (1); sana crítica (4); indicios/prueba indiciaria (1)</t>
         </is>
       </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3473,6 +3714,11 @@
           <t>valoración probatoria (2); apreciación probatoria (1); sana crítica (6); indicios/prueba indiciaria (2)</t>
         </is>
       </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3535,6 +3781,11 @@
           <t>valoración probatoria (4); indicios/prueba indiciaria (1)</t>
         </is>
       </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3597,6 +3848,11 @@
           <t>valoración probatoria (5); sana crítica (4); indicios/prueba indiciaria (3)</t>
         </is>
       </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3659,6 +3915,11 @@
           <t>valoración probatoria (4); sana crítica (1)</t>
         </is>
       </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3717,6 +3978,11 @@
           <t>valoración probatoria (1); apreciación probatoria (1); sana crítica (3); indicios/prueba indiciaria (1); prueba trasladada (6)</t>
         </is>
       </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>Título sin radicado completo; no comparable</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3779,6 +4045,11 @@
           <t>valoración probatoria (1); sana crítica (2); prueba ilícita/exclusión (6); indicios/prueba indiciaria (7)</t>
         </is>
       </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3841,6 +4112,11 @@
           <t>valoración probatoria (11); apreciación probatoria (3); sana crítica (9); indicios/prueba indiciaria (1); prueba trasladada (1)</t>
         </is>
       </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3903,6 +4179,11 @@
           <t>valoración probatoria (3); sana crítica (2)</t>
         </is>
       </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3965,6 +4246,11 @@
           <t>valoración probatoria (1); sana crítica (1)</t>
         </is>
       </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4027,6 +4313,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4089,6 +4380,11 @@
           <t>valoración probatoria (3); indicios/prueba indiciaria (1)</t>
         </is>
       </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4151,6 +4447,11 @@
           <t>valoración probatoria (2); sana crítica (1); prueba ilícita/exclusión (3)</t>
         </is>
       </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4213,6 +4514,11 @@
           <t>valoración probatoria (1); sana crítica (1)</t>
         </is>
       </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4275,6 +4581,11 @@
           <t>sana crítica (1)</t>
         </is>
       </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4337,6 +4648,11 @@
           <t>valoración probatoria (3)</t>
         </is>
       </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4399,6 +4715,11 @@
           <t>sana crítica (1)</t>
         </is>
       </c>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4461,6 +4782,11 @@
           <t>sana crítica (3)</t>
         </is>
       </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4523,6 +4849,11 @@
           <t>sana crítica (1)</t>
         </is>
       </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4585,6 +4916,11 @@
           <t>valoración probatoria (1); sana crítica (4)</t>
         </is>
       </c>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4647,6 +4983,11 @@
           <t>valoración probatoria (5); sana crítica (3)</t>
         </is>
       </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4709,6 +5050,11 @@
           <t>valoración probatoria (5); sana crítica (3)</t>
         </is>
       </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4771,6 +5117,11 @@
           <t>valoración probatoria (2); indicios/prueba indiciaria (12)</t>
         </is>
       </c>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>Título sin radicado completo; no comparable</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4833,6 +5184,11 @@
           <t>valoración probatoria (6); sana crítica (4)</t>
         </is>
       </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4895,6 +5251,11 @@
           <t>valoración probatoria (6); sana crítica (4)</t>
         </is>
       </c>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>Título sin radicado completo; no comparable</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4957,6 +5318,11 @@
           <t>valoración probatoria (1); sana crítica (1)</t>
         </is>
       </c>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5019,6 +5385,11 @@
           <t>valoración probatoria (1); sana crítica (2)</t>
         </is>
       </c>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -5081,6 +5452,11 @@
           <t>valoración probatoria (2); sana crítica (2)</t>
         </is>
       </c>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5143,6 +5519,11 @@
           <t>sana crítica (1)</t>
         </is>
       </c>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -5205,6 +5586,11 @@
           <t>valoración probatoria (2); sana crítica (1)</t>
         </is>
       </c>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -5267,6 +5653,11 @@
           <t>valoración probatoria (5); sana crítica (1)</t>
         </is>
       </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -5329,6 +5720,11 @@
           <t>valoración probatoria (3); sana crítica (1)</t>
         </is>
       </c>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -5391,6 +5787,11 @@
           <t>sana crítica (1); indicios/prueba indiciaria (2)</t>
         </is>
       </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5453,6 +5854,11 @@
           <t>valoración probatoria (4)</t>
         </is>
       </c>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5515,6 +5921,11 @@
           <t>valoración probatoria (4)</t>
         </is>
       </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -5577,6 +5988,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -5639,6 +6055,11 @@
           <t>valoración probatoria (2); sana crítica (2)</t>
         </is>
       </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -5701,6 +6122,11 @@
           <t>valoración probatoria (1); sana crítica (1)</t>
         </is>
       </c>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5763,6 +6189,11 @@
           <t>valoración probatoria (2); sana crítica (2)</t>
         </is>
       </c>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -5825,6 +6256,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5887,6 +6323,11 @@
           <t>valoración probatoria (1); indicios/prueba indiciaria (4)</t>
         </is>
       </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -5949,6 +6390,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -6011,6 +6457,11 @@
           <t>valoración probatoria (3); sana crítica (1)</t>
         </is>
       </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -6073,6 +6524,11 @@
           <t>valoración probatoria (1); indicios/prueba indiciaria (3)</t>
         </is>
       </c>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -6135,6 +6591,11 @@
           <t>sana crítica (1)</t>
         </is>
       </c>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -6197,6 +6658,11 @@
           <t>sana crítica (1); indicios/prueba indiciaria (1)</t>
         </is>
       </c>
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -6257,6 +6723,11 @@
       <c r="L94" s="2" t="inlineStr">
         <is>
           <t>valoración probatoria (5); sana crítica (1)</t>
+        </is>
+      </c>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
         </is>
       </c>
     </row>
@@ -6313,6 +6784,11 @@
           <t>sana crítica (1)</t>
         </is>
       </c>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>Título sin radicado completo; no comparable</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -6375,6 +6851,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>Título sin radicado completo; no comparable</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -6437,6 +6918,11 @@
           <t>valoración probatoria (2); sana crítica (6)</t>
         </is>
       </c>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>Título sin radicado completo; no comparable</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -6499,6 +6985,11 @@
           <t>sana crítica (1); indicios/prueba indiciaria (4); prueba trasladada (2)</t>
         </is>
       </c>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -6561,6 +7052,11 @@
           <t>ninguno de los 6 términos aparece en el texto</t>
         </is>
       </c>
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -6623,6 +7119,11 @@
           <t>ninguno de los 6 términos</t>
         </is>
       </c>
+      <c r="M100" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -6685,6 +7186,11 @@
           <t>ninguno de los 6 términos</t>
         </is>
       </c>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -6747,6 +7253,11 @@
           <t>sana crítica (1); indicios/prueba indiciaria (1)</t>
         </is>
       </c>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -6809,6 +7320,11 @@
           <t>sana crítica (1)</t>
         </is>
       </c>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -6871,6 +7387,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -6933,6 +7454,11 @@
           <t>indicios/prueba indiciaria (1)</t>
         </is>
       </c>
+      <c r="M105" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -6995,6 +7521,11 @@
           <t>indicios/prueba indiciaria (3)</t>
         </is>
       </c>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -7057,6 +7588,11 @@
           <t>sana crítica (1)</t>
         </is>
       </c>
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -7119,6 +7655,11 @@
           <t>ninguno de los 6 términos</t>
         </is>
       </c>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -7181,6 +7722,11 @@
           <t>sana crítica (1)</t>
         </is>
       </c>
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -7243,6 +7789,11 @@
           <t>sana crítica (1)</t>
         </is>
       </c>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -7305,6 +7856,11 @@
           <t>valoración probatoria (1); indicios/prueba indiciaria (1)</t>
         </is>
       </c>
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -7367,6 +7923,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -7429,6 +7990,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M113" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -7491,6 +8057,11 @@
           <t>valoración probatoria (1); sana crítica (2)</t>
         </is>
       </c>
+      <c r="M114" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -7553,6 +8124,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M115" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -7615,6 +8191,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M116" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -7677,6 +8258,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M117" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -7739,6 +8325,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>Título sin radicado completo; no comparable</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -7801,6 +8392,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M119" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -7863,6 +8459,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -7925,6 +8526,11 @@
           <t>ninguno de los 6 términos</t>
         </is>
       </c>
+      <c r="M121" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -7987,6 +8593,11 @@
           <t>valoración probatoria (1); sana crítica (1)</t>
         </is>
       </c>
+      <c r="M122" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -8049,6 +8660,11 @@
           <t>valoración probatoria (2); sana crítica (1)</t>
         </is>
       </c>
+      <c r="M123" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -8111,6 +8727,11 @@
           <t>ninguno de los 6 términos</t>
         </is>
       </c>
+      <c r="M124" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -8173,6 +8794,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M125" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -8235,6 +8861,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M126" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -8297,6 +8928,11 @@
           <t>valoración probatoria (1); sana crítica (1)</t>
         </is>
       </c>
+      <c r="M127" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -8359,6 +8995,11 @@
           <t>ninguno de los 6 términos</t>
         </is>
       </c>
+      <c r="M128" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -8421,6 +9062,11 @@
           <t>ninguno de los 6 términos</t>
         </is>
       </c>
+      <c r="M129" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -8483,6 +9129,11 @@
           <t>ninguno de los 6 términos</t>
         </is>
       </c>
+      <c r="M130" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -8545,6 +9196,11 @@
           <t>sana crítica (1)</t>
         </is>
       </c>
+      <c r="M131" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -8607,6 +9263,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M132" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -8669,6 +9330,11 @@
           <t>indicios/prueba indiciaria (1)</t>
         </is>
       </c>
+      <c r="M133" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -8731,6 +9397,11 @@
           <t>ninguno de los 6 términos</t>
         </is>
       </c>
+      <c r="M134" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -8793,6 +9464,11 @@
           <t>ninguno de los 6 términos</t>
         </is>
       </c>
+      <c r="M135" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -8855,6 +9531,11 @@
           <t>indicios/prueba indiciaria (1)</t>
         </is>
       </c>
+      <c r="M136" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -8917,6 +9598,11 @@
           <t>indicios/prueba indiciaria (1)</t>
         </is>
       </c>
+      <c r="M137" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -8979,6 +9665,11 @@
           <t>valoración probatoria (2)</t>
         </is>
       </c>
+      <c r="M138" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -9041,6 +9732,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M139" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -9103,6 +9799,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M140" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -9165,6 +9866,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M141" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -9227,6 +9933,11 @@
           <t>sana crítica (1)</t>
         </is>
       </c>
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -9289,6 +10000,11 @@
           <t>ninguno de los 6 términos</t>
         </is>
       </c>
+      <c r="M143" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -9351,6 +10067,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M144" s="2" t="inlineStr">
+        <is>
+          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -9413,6 +10134,11 @@
           <t>sana crítica (1)</t>
         </is>
       </c>
+      <c r="M145" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -9475,6 +10201,11 @@
           <t>ninguno de los 6 términos</t>
         </is>
       </c>
+      <c r="M146" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -9537,6 +10268,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M147" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -9599,6 +10335,11 @@
           <t>indicios/prueba indiciaria (1)</t>
         </is>
       </c>
+      <c r="M148" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -9659,6 +10400,11 @@
       <c r="L149" s="2" t="inlineStr">
         <is>
           <t>valoración probatoria (1)</t>
+        </is>
+      </c>
+      <c r="M149" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
         </is>
       </c>
     </row>
@@ -9715,6 +10461,11 @@
           <t>ninguno de los 6 términos</t>
         </is>
       </c>
+      <c r="M150" s="2" t="inlineStr">
+        <is>
+          <t>Título sin radicado completo; no comparable</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -9777,6 +10528,11 @@
           <t>valoración probatoria (1); sana crítica (1)</t>
         </is>
       </c>
+      <c r="M151" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -9839,6 +10595,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M152" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -9901,6 +10662,11 @@
           <t>valoración probatoria (1)</t>
         </is>
       </c>
+      <c r="M153" s="2" t="inlineStr">
+        <is>
+          <t>Confirmado en el encabezado</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -9955,6 +10721,11 @@
       </c>
       <c r="K154" s="2" t="n"/>
       <c r="L154" s="2" t="n"/>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -10009,6 +10780,11 @@
       </c>
       <c r="K155" s="2" t="n"/>
       <c r="L155" s="2" t="n"/>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -10063,6 +10839,11 @@
       </c>
       <c r="K156" s="2" t="n"/>
       <c r="L156" s="2" t="n"/>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -10117,6 +10898,11 @@
       </c>
       <c r="K157" s="2" t="n"/>
       <c r="L157" s="2" t="n"/>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -10167,6 +10953,11 @@
       </c>
       <c r="K158" s="2" t="n"/>
       <c r="L158" s="2" t="n"/>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -10213,6 +11004,11 @@
       </c>
       <c r="K159" s="2" t="n"/>
       <c r="L159" s="2" t="n"/>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -10259,6 +11055,11 @@
       </c>
       <c r="K160" s="2" t="n"/>
       <c r="L160" s="2" t="n"/>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -10309,6 +11110,11 @@
       </c>
       <c r="K161" s="2" t="n"/>
       <c r="L161" s="2" t="n"/>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -10363,6 +11169,11 @@
       </c>
       <c r="K162" s="2" t="n"/>
       <c r="L162" s="2" t="n"/>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -10417,6 +11228,11 @@
       </c>
       <c r="K163" s="2" t="n"/>
       <c r="L163" s="2" t="n"/>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -10471,6 +11287,11 @@
       </c>
       <c r="K164" s="2" t="n"/>
       <c r="L164" s="2" t="n"/>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -10525,6 +11346,11 @@
       </c>
       <c r="K165" s="2" t="n"/>
       <c r="L165" s="2" t="n"/>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -10579,6 +11405,11 @@
       </c>
       <c r="K166" s="2" t="n"/>
       <c r="L166" s="2" t="n"/>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -10633,6 +11464,11 @@
       </c>
       <c r="K167" s="2" t="n"/>
       <c r="L167" s="2" t="n"/>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -10687,6 +11523,11 @@
       </c>
       <c r="K168" s="2" t="n"/>
       <c r="L168" s="2" t="n"/>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -10741,6 +11582,11 @@
       </c>
       <c r="K169" s="2" t="n"/>
       <c r="L169" s="2" t="n"/>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -10795,6 +11641,11 @@
       </c>
       <c r="K170" s="2" t="n"/>
       <c r="L170" s="2" t="n"/>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -10849,6 +11700,11 @@
       </c>
       <c r="K171" s="2" t="n"/>
       <c r="L171" s="2" t="n"/>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -10903,6 +11759,11 @@
       </c>
       <c r="K172" s="2" t="n"/>
       <c r="L172" s="2" t="n"/>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -10957,6 +11818,11 @@
       </c>
       <c r="K173" s="2" t="n"/>
       <c r="L173" s="2" t="n"/>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -11011,6 +11877,11 @@
       </c>
       <c r="K174" s="2" t="n"/>
       <c r="L174" s="2" t="n"/>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -11065,6 +11936,11 @@
       </c>
       <c r="K175" s="2" t="n"/>
       <c r="L175" s="2" t="n"/>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -11119,6 +11995,11 @@
       </c>
       <c r="K176" s="2" t="n"/>
       <c r="L176" s="2" t="n"/>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
@@ -11173,6 +12054,11 @@
       </c>
       <c r="K177" s="2" t="n"/>
       <c r="L177" s="2" t="n"/>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -11227,6 +12113,11 @@
       </c>
       <c r="K178" s="2" t="n"/>
       <c r="L178" s="2" t="n"/>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -11281,6 +12172,11 @@
       </c>
       <c r="K179" s="2" t="n"/>
       <c r="L179" s="2" t="n"/>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -11335,6 +12231,11 @@
       </c>
       <c r="K180" s="2" t="n"/>
       <c r="L180" s="2" t="n"/>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -11389,6 +12290,11 @@
       </c>
       <c r="K181" s="2" t="n"/>
       <c r="L181" s="2" t="n"/>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -11439,6 +12345,11 @@
       </c>
       <c r="K182" s="2" t="n"/>
       <c r="L182" s="2" t="n"/>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -11489,6 +12400,11 @@
       </c>
       <c r="K183" s="2" t="n"/>
       <c r="L183" s="2" t="n"/>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -11543,6 +12459,11 @@
       </c>
       <c r="K184" s="2" t="n"/>
       <c r="L184" s="2" t="n"/>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
@@ -11597,6 +12518,11 @@
       </c>
       <c r="K185" s="2" t="n"/>
       <c r="L185" s="2" t="n"/>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -11651,6 +12577,11 @@
       </c>
       <c r="K186" s="2" t="n"/>
       <c r="L186" s="2" t="n"/>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
@@ -11705,6 +12636,11 @@
       </c>
       <c r="K187" s="2" t="n"/>
       <c r="L187" s="2" t="n"/>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -11759,6 +12695,11 @@
       </c>
       <c r="K188" s="2" t="n"/>
       <c r="L188" s="2" t="n"/>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
@@ -11813,6 +12754,11 @@
       </c>
       <c r="K189" s="2" t="n"/>
       <c r="L189" s="2" t="n"/>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -11867,6 +12813,11 @@
       </c>
       <c r="K190" s="2" t="n"/>
       <c r="L190" s="2" t="n"/>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
@@ -11921,6 +12872,11 @@
       </c>
       <c r="K191" s="2" t="n"/>
       <c r="L191" s="2" t="n"/>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -11975,6 +12931,11 @@
       </c>
       <c r="K192" s="2" t="n"/>
       <c r="L192" s="2" t="n"/>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -12029,6 +12990,11 @@
       </c>
       <c r="K193" s="2" t="n"/>
       <c r="L193" s="2" t="n"/>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -12083,6 +13049,11 @@
       </c>
       <c r="K194" s="2" t="n"/>
       <c r="L194" s="2" t="n"/>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -12137,6 +13108,11 @@
       </c>
       <c r="K195" s="2" t="n"/>
       <c r="L195" s="2" t="n"/>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -12191,6 +13167,11 @@
       </c>
       <c r="K196" s="2" t="n"/>
       <c r="L196" s="2" t="n"/>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
@@ -12245,6 +13226,11 @@
       </c>
       <c r="K197" s="2" t="n"/>
       <c r="L197" s="2" t="n"/>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -12299,6 +13285,11 @@
       </c>
       <c r="K198" s="2" t="n"/>
       <c r="L198" s="2" t="n"/>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
@@ -12353,6 +13344,11 @@
       </c>
       <c r="K199" s="2" t="n"/>
       <c r="L199" s="2" t="n"/>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -12407,6 +13403,11 @@
       </c>
       <c r="K200" s="2" t="n"/>
       <c r="L200" s="2" t="n"/>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
@@ -12461,6 +13462,11 @@
       </c>
       <c r="K201" s="2" t="n"/>
       <c r="L201" s="2" t="n"/>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -12515,6 +13521,11 @@
       </c>
       <c r="K202" s="2" t="n"/>
       <c r="L202" s="2" t="n"/>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
@@ -12569,6 +13580,11 @@
       </c>
       <c r="K203" s="2" t="n"/>
       <c r="L203" s="2" t="n"/>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -12623,6 +13639,11 @@
       </c>
       <c r="K204" s="2" t="n"/>
       <c r="L204" s="2" t="n"/>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
@@ -12677,6 +13698,11 @@
       </c>
       <c r="K205" s="2" t="n"/>
       <c r="L205" s="2" t="n"/>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -12731,6 +13757,11 @@
       </c>
       <c r="K206" s="2" t="n"/>
       <c r="L206" s="2" t="n"/>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
@@ -12785,6 +13816,11 @@
       </c>
       <c r="K207" s="2" t="n"/>
       <c r="L207" s="2" t="n"/>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -12839,6 +13875,11 @@
       </c>
       <c r="K208" s="2" t="n"/>
       <c r="L208" s="2" t="n"/>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
@@ -12893,6 +13934,11 @@
       </c>
       <c r="K209" s="2" t="n"/>
       <c r="L209" s="2" t="n"/>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -12947,6 +13993,11 @@
       </c>
       <c r="K210" s="2" t="n"/>
       <c r="L210" s="2" t="n"/>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
@@ -13001,6 +14052,11 @@
       </c>
       <c r="K211" s="2" t="n"/>
       <c r="L211" s="2" t="n"/>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
@@ -13055,6 +14111,11 @@
       </c>
       <c r="K212" s="2" t="n"/>
       <c r="L212" s="2" t="n"/>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
@@ -13109,6 +14170,11 @@
       </c>
       <c r="K213" s="2" t="n"/>
       <c r="L213" s="2" t="n"/>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
@@ -13163,6 +14229,11 @@
       </c>
       <c r="K214" s="2" t="n"/>
       <c r="L214" s="2" t="n"/>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
@@ -13217,6 +14288,11 @@
       </c>
       <c r="K215" s="2" t="n"/>
       <c r="L215" s="2" t="n"/>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
@@ -13271,6 +14347,11 @@
       </c>
       <c r="K216" s="2" t="n"/>
       <c r="L216" s="2" t="n"/>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
@@ -13325,6 +14406,11 @@
       </c>
       <c r="K217" s="2" t="n"/>
       <c r="L217" s="2" t="n"/>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
@@ -13379,6 +14465,11 @@
       </c>
       <c r="K218" s="2" t="n"/>
       <c r="L218" s="2" t="n"/>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
@@ -13433,6 +14524,11 @@
       </c>
       <c r="K219" s="2" t="n"/>
       <c r="L219" s="2" t="n"/>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -13487,6 +14583,11 @@
       </c>
       <c r="K220" s="2" t="n"/>
       <c r="L220" s="2" t="n"/>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
@@ -13541,6 +14642,11 @@
       </c>
       <c r="K221" s="2" t="n"/>
       <c r="L221" s="2" t="n"/>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
@@ -13595,6 +14701,11 @@
       </c>
       <c r="K222" s="2" t="n"/>
       <c r="L222" s="2" t="n"/>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
@@ -13649,6 +14760,11 @@
       </c>
       <c r="K223" s="2" t="n"/>
       <c r="L223" s="2" t="n"/>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
@@ -13703,6 +14819,11 @@
       </c>
       <c r="K224" s="2" t="n"/>
       <c r="L224" s="2" t="n"/>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
@@ -13757,6 +14878,11 @@
       </c>
       <c r="K225" s="2" t="n"/>
       <c r="L225" s="2" t="n"/>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
@@ -13807,6 +14933,11 @@
       </c>
       <c r="K226" s="2" t="n"/>
       <c r="L226" s="2" t="n"/>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
@@ -13861,6 +14992,11 @@
       </c>
       <c r="K227" s="2" t="n"/>
       <c r="L227" s="2" t="n"/>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
@@ -13915,6 +15051,11 @@
       </c>
       <c r="K228" s="2" t="n"/>
       <c r="L228" s="2" t="n"/>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
@@ -13969,6 +15110,11 @@
       </c>
       <c r="K229" s="2" t="n"/>
       <c r="L229" s="2" t="n"/>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
@@ -14023,6 +15169,11 @@
       </c>
       <c r="K230" s="2" t="n"/>
       <c r="L230" s="2" t="n"/>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
@@ -14077,6 +15228,11 @@
       </c>
       <c r="K231" s="2" t="n"/>
       <c r="L231" s="2" t="n"/>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
@@ -14131,6 +15287,11 @@
       </c>
       <c r="K232" s="2" t="n"/>
       <c r="L232" s="2" t="n"/>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
@@ -14181,6 +15342,11 @@
       </c>
       <c r="K233" s="2" t="n"/>
       <c r="L233" s="2" t="n"/>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
@@ -14235,6 +15401,11 @@
       </c>
       <c r="K234" s="2" t="n"/>
       <c r="L234" s="2" t="n"/>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
@@ -14285,6 +15456,11 @@
       </c>
       <c r="K235" s="2" t="n"/>
       <c r="L235" s="2" t="n"/>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
@@ -14339,6 +15515,11 @@
       </c>
       <c r="K236" s="2" t="n"/>
       <c r="L236" s="2" t="n"/>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
@@ -14385,6 +15566,11 @@
       </c>
       <c r="K237" s="2" t="n"/>
       <c r="L237" s="2" t="n"/>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
@@ -14431,6 +15617,11 @@
       </c>
       <c r="K238" s="2" t="n"/>
       <c r="L238" s="2" t="n"/>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
@@ -14477,6 +15668,11 @@
       </c>
       <c r="K239" s="2" t="n"/>
       <c r="L239" s="2" t="n"/>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
@@ -14523,6 +15719,11 @@
       </c>
       <c r="K240" s="2" t="n"/>
       <c r="L240" s="2" t="n"/>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
@@ -14577,6 +15778,11 @@
       </c>
       <c r="K241" s="2" t="n"/>
       <c r="L241" s="2" t="n"/>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
@@ -14631,6 +15837,11 @@
       </c>
       <c r="K242" s="2" t="n"/>
       <c r="L242" s="2" t="n"/>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
@@ -14685,6 +15896,11 @@
       </c>
       <c r="K243" s="2" t="n"/>
       <c r="L243" s="2" t="n"/>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
@@ -14739,6 +15955,11 @@
       </c>
       <c r="K244" s="2" t="n"/>
       <c r="L244" s="2" t="n"/>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
@@ -14793,6 +16014,11 @@
       </c>
       <c r="K245" s="2" t="n"/>
       <c r="L245" s="2" t="n"/>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
@@ -14847,6 +16073,11 @@
       </c>
       <c r="K246" s="2" t="n"/>
       <c r="L246" s="2" t="n"/>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
@@ -14901,6 +16132,11 @@
       </c>
       <c r="K247" s="2" t="n"/>
       <c r="L247" s="2" t="n"/>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
@@ -14955,6 +16191,11 @@
       </c>
       <c r="K248" s="2" t="n"/>
       <c r="L248" s="2" t="n"/>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
@@ -15009,6 +16250,11 @@
       </c>
       <c r="K249" s="2" t="n"/>
       <c r="L249" s="2" t="n"/>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
@@ -15063,6 +16309,11 @@
       </c>
       <c r="K250" s="2" t="n"/>
       <c r="L250" s="2" t="n"/>
+      <c r="M250" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
@@ -15117,6 +16368,11 @@
       </c>
       <c r="K251" s="2" t="n"/>
       <c r="L251" s="2" t="n"/>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
@@ -15167,6 +16423,11 @@
       </c>
       <c r="K252" s="2" t="n"/>
       <c r="L252" s="2" t="n"/>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
@@ -15213,6 +16474,11 @@
       </c>
       <c r="K253" s="2" t="n"/>
       <c r="L253" s="2" t="n"/>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
@@ -15267,6 +16533,11 @@
       </c>
       <c r="K254" s="2" t="n"/>
       <c r="L254" s="2" t="n"/>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
@@ -15321,6 +16592,11 @@
       </c>
       <c r="K255" s="2" t="n"/>
       <c r="L255" s="2" t="n"/>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
@@ -15375,6 +16651,11 @@
       </c>
       <c r="K256" s="2" t="n"/>
       <c r="L256" s="2" t="n"/>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
@@ -15429,6 +16710,11 @@
       </c>
       <c r="K257" s="2" t="n"/>
       <c r="L257" s="2" t="n"/>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
@@ -15483,6 +16769,11 @@
       </c>
       <c r="K258" s="2" t="n"/>
       <c r="L258" s="2" t="n"/>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
@@ -15537,6 +16828,11 @@
       </c>
       <c r="K259" s="2" t="n"/>
       <c r="L259" s="2" t="n"/>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
@@ -15591,6 +16887,11 @@
       </c>
       <c r="K260" s="2" t="n"/>
       <c r="L260" s="2" t="n"/>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>No leída</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L260"/>
@@ -15604,7 +16905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -15666,6 +16967,13 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Auditoría de radicados (col. M): 105 confirmados en el encabezado, 4 en el texto completo, 3 desajustes de título confirmados (archivo contiene otra sentencia ya incluida en la matriz), 33 no confirmados por tener encabezado de relatoría sin radicado, 11 sin radicado comparable en el título.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Completar verificación de radicados de las 29 providencias pendientes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HFz41Xq5pxE4jPsKEtG9Mg
</commit_message>
<xml_diff>
--- a/Matriz_Valoracion_Probatoria_Disciplinaria.xlsx
+++ b/Matriz_Valoracion_Probatoria_Disciplinaria.xlsx
@@ -1727,7 +1727,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>0051-2013</t>
+          <t>11001-03-25-000-2013-00017-00 (0051-2013)</t>
         </is>
       </c>
       <c r="D20" s="2" t="n"/>
@@ -1773,7 +1773,7 @@
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente); radicado propio: 11001-03-25-000-2013-00017-00 (0051-2013)</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -2309,7 +2309,7 @@
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -2510,7 +2510,7 @@
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -2778,7 +2778,7 @@
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -4784,7 +4784,7 @@
       </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
       </c>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -4985,7 +4985,7 @@
       </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -5186,7 +5186,7 @@
       </c>
       <c r="M71" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -6987,7 +6987,7 @@
       </c>
       <c r="M98" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente); radicado propio: 2018-00394 (None)</t>
         </is>
       </c>
     </row>
@@ -7657,7 +7657,7 @@
       </c>
       <c r="M108" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -7724,7 +7724,7 @@
       </c>
       <c r="M109" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="M111" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -7925,7 +7925,7 @@
       </c>
       <c r="M112" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -7992,7 +7992,7 @@
       </c>
       <c r="M113" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -8193,7 +8193,7 @@
       </c>
       <c r="M116" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -8260,7 +8260,7 @@
       </c>
       <c r="M117" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -8394,7 +8394,7 @@
       </c>
       <c r="M119" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -9550,7 +9550,7 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>1093-2013</t>
+          <t>11001-03-25-000-2013-00561-00 (1093-2013)</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -9600,7 +9600,7 @@
       </c>
       <c r="M137" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente); radicado propio: 11001-03-25-000-2013-00561-00 (1093-2013)</t>
         </is>
       </c>
     </row>
@@ -9684,7 +9684,7 @@
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>0552-2021</t>
+          <t>15001-2333-000-2017-00604-01 (0552-2021)</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="M139" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente); radicado propio: 15001-2333-000-2017-00604-01 (0552-2021)</t>
         </is>
       </c>
     </row>
@@ -10069,7 +10069,7 @@
       </c>
       <c r="M144" s="2" t="inlineStr">
         <is>
-          <t>No confirmado: el encabezado del texto no trae radicado (suele iniciar con relatoría); revisar</t>
+          <t>Confirmado en el texto completo (lectura por subagente)</t>
         </is>
       </c>
     </row>
@@ -16970,7 +16970,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Auditoría de radicados (col. M): 105 confirmados en el encabezado, 4 en el texto completo, 3 desajustes de título confirmados (el archivo contiene otra sentencia ya incluida en la matriz), 29 no confirmados por tener encabezado de relatoría sin radicado, 11 sin radicado comparable en el título.</t>
+          <t>Auditoría de radicados (col. M): 105 confirmados en el encabezado; 33 confirmados en el texto completo (4 por la asistente y 29 por subagentes); 3 desajustes de título confirmados (el archivo contiene otra sentencia ya incluida en la matriz); 11 sin radicado comparable en el título.</t>
         </is>
       </c>
     </row>

</xml_diff>